<commit_message>
Golden Path Slab: full re-run on v109.24 (51 slabs with saw loss, per-lot cost, thickness columns), green 'changed this round' flags
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/client-docs/test-cases/emg-o-golden-path-slab-cut-to-scrap.xlsx
+++ b/client-docs/test-cases/emg-o-golden-path-slab-cut-to-scrap.xlsx
@@ -677,7 +677,7 @@
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>Quantity 2.7000 ลบ.ม., Unit Price 27,000.00, ยอดก่อน VAT 72,900.00, VAT 7% 5,103.00, รวม 78,003.00 บาท · หลัง Confirm มีปุ่มสมาร์ท Receipt 1 ใบ (ตัวอย่างจริง P00094)</t>
+          <t>Quantity 2.7000 ลบ.ม., Unit Price 27,000.00, ยอดก่อน VAT 72,900.00, VAT 7% 5,103.00, รวม 78,003.00 บาท · หลัง Confirm มีปุ่มสมาร์ท Receipt 1 ใบ (ตัวอย่างจริง P00308)</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -687,7 +687,8 @@
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>เลือกตันที่หาร 2.7 ลงตัว (7.29 ตัน = 2.70 ลบ.ม.) ราคาจะไม่เพี้ยนเศษสตางค์ · ตอนพิมพ์ชื่อสินค้า อย่ากดบรรทัด "Create ..." ใน dropdown เพราะจะสร้างสินค้าซ้ำ</t>
+          <t>[แก้/เพิ่ม] รอบ 14 ต.ค. 2569 (v109.24) — หน่วยและช่องเหมือนเดิม แต่ PO ใบนี้จะกลายเป็นบิลผู้ขายในหน่วยตัน (ดู Golden Path Block TC-GP-BPC-04)
+เลือกตันที่หาร 2.7 ลงตัว (7.29 ตัน = 2.70 ลบ.ม.) ราคาจะไม่เพี้ยนเศษสตางค์ · ตอนพิมพ์ชื่อสินค้า อย่ากดบรรทัด "Create ..." ใน dropdown เพราะจะสร้างสินค้าซ้ำ</t>
         </is>
       </c>
       <c r="I4" s="7" t="n"/>
@@ -714,19 +715,20 @@
       <c r="D5" s="7" t="inlineStr">
         <is>
           <t>1. ที่ PO กดปุ่ม Receipt เพื่อเปิดใบรับของ
-2. กดคำว่า Details ที่แถว Block แล้วกรอก ยาว / กว้าง / สูง ของก้อนที่รับ
+2. กดคำว่า Details ที่แถว Block แล้วกรอก ยาว / กว้าง / สูง และ ตันตามใบส่งของ ของก้อนที่รับ
 3. กด Save แล้วกด Validate
 4. เปิดแอป Stone Slab &gt; Blocks ค้นหา Block ใหม่ แล้วดูการ์ดสรุปด้านบน</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>ขนาด Block = 2.50 × 1.20 × 0.90 ม.</t>
+          <t>ขนาด Block = 2.50 × 1.20 × 0.90 ม.
+ตันตามใบส่งของ = 7.300 ตัน</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>ใบรับของเป็น Done, Quantity 2.70 เท่ากับที่สั่ง จึงไม่มี Backorder · ได้ Block ใหม่ 1 ก้อน (ตัวอย่างจริง BLK-26-0037) สถานะ "ใช้ได้" ขนาด 2.50 × 1.20 × 0.90 = 2.70 CBM · 7.29 ตัน ต้นทุน 10,000 บาท/ตัน (27,000 บาท/CBM) อ้างอิง PO P00094 ผลการตัด "ยังไม่ได้ตัด"</t>
+          <t>ใบรับของเป็น Done (EG01/IN/00376), Quantity 2.70 เท่ากับที่สั่ง จึงไม่มี Backorder · ได้ Block ใหม่ 1 ก้อน (ตัวอย่างจริง BLK-26-0431) สถานะ "ใช้ได้" ขนาด 2.50 × 1.20 × 0.90 = 2.70 CBM · 7.30 ตัน ต้นทุน 10,000 บาท/ตัน (27,000 บาท/CBM) อ้างอิง PO P00308 % สูญเสียที่ใช้ 15.00 ผลการตัด "ยังไม่ได้ตัด"</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -736,7 +738,8 @@
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>การ์ด Block แสดง "ประมาณ 28 แผ่น / 135.00 ตร.ม." ตร.ม. รวมตรงกับที่ตัดจริง แต่จำนวนแผ่นต่างจากใบสั่งตัด (60 แผ่น) เพราะการ์ดประมาณจากขนาด Slab มาตรฐานของวัสดุ ไม่ได้ดูรูปทรงก้อนนี้ — ใช้เลขในใบสั่งตัดเป็นหลัก</t>
+          <t>[แก้/เพิ่ม] รอบ 14 ต.ค. 2569 (v109.24) — ใบรับของมีช่อง "ตันตามใบส่งของ" (ตัวอย่างนี้ 7.300 ตัน) ตันนี้กลายเป็นตันของ Block และใช้คิดต้นทุน · การ์ด Block มีส่วน "% สูญเสียจากการเลื่อย" (15%) และช่อง QC Note
+การ์ด Block แสดง "ประมาณ 28 แผ่น / 135.00 ตร.ม." ซึ่งเป็นค่าประมาณจากขนาด Slab มาตรฐานของวัสดุ ไม่ตรงกับจำนวนแผ่นในใบสั่งตัด (51 แผ่น) — ใช้เลขในใบสั่งตัดเป็นหลัก · ตันตามใบส่งของเว้นว่างได้ ระบบจะใช้ ลบ.ม. × 2.7 แทน</t>
         </is>
       </c>
       <c r="I5" s="7" t="n"/>
@@ -871,7 +874,7 @@
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>Block = BLK-26-0037
+          <t>Block = BLK-26-0431
 Finish = Polished
 Thickness = 2 cm
 เหตุผล = งานเพิ่ม (Extra work)</t>
@@ -879,7 +882,7 @@
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>การ์ดบนหน้าแสดง Block ที่ตัด BLK-26-0037 เหลือ 2.70 CBM · ขนาดเป้าหมาย 2.50 × 0.90 ม. Polished หนา 0.02 ม. · ความคืบหน้า ประมาณ 60 แผ่น = 135.00 ตร.ม. · "จะได้ Slab: ... Slab (Polished, 2 cm)" · แท็บ "Slab ที่ตัดได้ (แผน/จริง)" มีแผน 60 แถว (หน้าละ 40 แถว) · มีแถบเหลืองบอกให้กด "ย้ายไปสถานีตัด" ก่อน Confirm</t>
+          <t>การ์ดบนหน้าแสดง Block ที่ตัด BLK-26-0431 เหลือ 2.70 CBM · ขนาดเป้าหมาย 2.50 × 0.90 ม. Polished หนา 0.02 ม. · ความคืบหน้า ประมาณ 51 แผ่น = 114.75 ตร.ม. · "จะได้ Slab: ... Slab (Polished, 2 cm)" · ข้อความเขียว "แผนใช้ 2.70 CBM (รวมสูญเสียเลื่อย 15%) พอ" · แท็บ "Slab ที่ตัดได้ (แผน/จริง)" มีแผน 51 แถว · มีแถบเหลืองบอกให้กด "ย้ายไปสถานีตัด" ก่อน Confirm (ตัวอย่างจริง EG01/STCUT/00229)</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -889,7 +892,8 @@
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>ใบสั่งตัดที่ยังเป็น Draft แท็บ Components อาจแสดง "60.00 m³ Not Available" เป็นการคูณตามสูตรมาตรฐานของ Odoo ไม่ใช่ปริมาณที่ใช้จริง พอ Confirm จะกลับเป็น 2.70 ลบ.ม. · ถ้าไม่มี Sale Order ต้องเลือก "เหตุผล (กรณีไม่มี SO)" ก่อนจึงจะ Confirm ได้</t>
+          <t>[แก้/เพิ่ม] รอบ 14 ต.ค. 2569 (v109.24) — แผนหัก "% สูญเสียจากการเลื่อย" 15% แล้ว: 51 แผ่น / 114.75 ตร.ม. (รอบ 11 ต.ค. เป็น 60 แผ่น / 135.00 ตร.ม.) และข้อความสีเขียวบอกว่าแผนใช้ 2.70 CBM รวมสูญเสียเลื่อยแล้ว
+ใบสั่งตัดที่ยังเป็น Draft แท็บ Components อาจแสดงปริมาณ Block ตามสูตรมาตรฐานของ Odoo (เช่น 51.00 m³ Not Available) ไม่ใช่ปริมาณที่ใช้จริง พอ Confirm จะกลับเป็น 2.70 ลบ.ม. · ถ้าไม่มี Sale Order ต้องเลือก "เหตุผล (กรณีไม่มี SO)" ก่อนจึงจะ Confirm ได้</t>
         </is>
       </c>
       <c r="I4" s="7" t="n"/>
@@ -926,7 +930,7 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>ข้อความ "ย้ายสำเร็จ (Moved). Block BLK-26-0037 ย้ายไป Stone Production แล้ว 2.700 หน่วย — กด Confirm ได้เลย" · หลัง Confirm ปุ่มเปลี่ยนเป็น "ตัดเสร็จ", Component Status = Available, ผู้รับผิดชอบเป็นผู้ใช้ปัจจุบัน (ตัวอย่างจริง EG01/STCUT/00050)</t>
+          <t>ข้อความ "ย้ายสำเร็จ (Moved). Block BLK-26-0431 ย้ายไป Stone Production แล้ว 2.700 หน่วย — กด Confirm ได้เลย" · หลัง Confirm ปุ่มเปลี่ยนเป็น "ตัดเสร็จ", Component Status = Available, ผู้รับผิดชอบเป็นผู้ใช้ปัจจุบัน (EG01/STCUT/00229)</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -962,7 +966,7 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>1. เปิดแท็บ "Slab ที่ตัดได้ (แผน/จริง)" ดูว่าแผนมี 60 แถว
+          <t>1. เปิดแท็บ "Slab ที่ตัดได้ (แผน/จริง)" ดูว่าแผนมี 51 แถว
 2. กดปุ่ม "ตัดเสร็จ"
 3. ดูแท็บ Slab อีกครั้ง และสมาร์ทปุ่ม Serial Numbers</t>
         </is>
@@ -974,7 +978,7 @@
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>ข้อความ "Complete Cut สำเร็จ ... ตัดได้ 60 แผ่นจาก BLK-26-0037" · สถานะ Done · Serial Numbers 60 · 60 แถวมีขนาดจริง 2.50 × 0.90 × 0.02 · การ์ดสรุป 135.00 ตร.ม. (100% ของแผน) · Block เหลือ 0 CBM · Slab BLK-26-0037-1 ถึง -60 สถานะ Available ต้นทุน 540 บาท/ตร.ม. (72,900 ÷ 135) ราคาขาย 4,000 บาท/ตร.ม.</t>
+          <t>ข้อความ "Complete Cut สำเร็จ ... ตัดได้ 51 แผ่นจาก BLK-26-0431" · สถานะ Done · Serial Numbers 51 · การ์ดสรุป 114.75 ตร.ม. (100% ของแผน) · Block เหลือ 0 CBM · Slab BLK-26-0431-1 ถึง -51 สถานะ Available ต้นทุนแผ่นละ 1,431.37 บาท (มูลค่าที่ย้ายจาก Block เป็น Slab 73,000.00 บาท) ราคาขาย 4,000 บาท/ตร.ม.</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
@@ -984,7 +988,8 @@
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>ชื่อ Slab ที่ตัดจาก Block ตั้งตามชื่อ Block (BLK-26-0037-1, -2, ...) ส่วน SLB-26-xxxx ใช้กับ Slab ที่ซื้อมาเป็นแผ่น · จำนวนแผ่นเป็นค่าสูงสุดตามทฤษฎี ยังไม่หักเนื้อหินที่หายไปกับใบเลื่อย</t>
+          <t>[แก้/เพิ่ม] รอบ 14 ต.ค. 2569 (v109.24) — ต้นทุนแผ่นแบ่งตามต้นทุนของ Block ก้อนนั้นเอง (7.30 ตัน × 10,000 = 73,000 บาท) หารจำนวนแผ่น 51 = 1,431.37 บาท/แผ่น (รอบ 11 ต.ค. คิด 540 บาท/ตร.ม. จาก 72,900 ÷ 135) เพราะแผนมีส่วนสูญเสียเลื่อยแล้ว
+ชื่อ Slab ที่ตัดจาก Block ตั้งตามชื่อ Block (BLK-26-0431-1, -2, ...) ส่วน SLB-26-xxxx ใช้กับ Slab ที่ซื้อมาเป็นแผ่น · Block ถูกใช้หมด (เหลือ 0 CBM) เพราะแผนรวมส่วนสูญเสียเลื่อยแล้ว</t>
         </is>
       </c>
       <c r="I6" s="7" t="n"/>
@@ -1120,12 +1125,12 @@
         <is>
           <t>ลูกค้า = Demo Hotel Customer
 Finish = Polished, Thickness = 2 cm
-เลือก BLK-26-0037-1 ถึง -10 (10 แผ่น)</t>
+เลือก BLK-26-0431-1 ถึง -10 (10 แผ่น)</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>บรรทัดสินค้าเป็น "10 แผ่น = 22.50 ตร.ม. · 4,000 ฿/ตร.ม." แสดงรายชื่อ 10 แผ่น แต่ละแผ่น 2.50 × 0.90 × 0.020 ม. = 2.25 ตร.ม. · Quantity 10.00 Units, Unit Price 9,000.00 (2.25 × 4,000) · สมาร์ทปุ่ม Slabs = 10 (ตัวอย่างจริง S00213)</t>
+          <t>บรรทัดสินค้าเป็น "10 แผ่น = 22.50 ตร.ม. · 4,000 ฿/ตร.ม." แสดงรายชื่อ 10 แผ่น แต่ละแผ่น 2.50 × 0.90 × 0.020 ม. = 2.25 ตร.ม. · หนา (ซม.) 2.00 · Quantity 10.00 Units, Unit Price 9,000.00 (2.25 × 4,000) · สมาร์ทปุ่ม Slabs = 10 (ตัวอย่างจริง S00625)</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -1133,7 +1138,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H4" s="7" t="n"/>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>[แก้/เพิ่ม] รอบ 14 ต.ค. 2569 (v109.24) — ใบขายมีคอลัมน์ "หนา (ซม.)" และ "เตือนกำไร" ราคาต่อ ตร.ม. ตามความหนา (ราคาตามตารางความหนาของวัสดุ) ภาพที่ 2 แสดงคอลัมน์เหล่านี้ (ปกติเป็นคอลัมน์เสริม เปิดได้จากไอคอนตั้งค่าท้ายหัวตาราง)
+ในภาพแรกซ่อนคอลัมน์เสริมเพื่อให้เห็นรายชื่อแผ่น</t>
+        </is>
+      </c>
       <c r="I4" s="7" t="n"/>
       <c r="J4" s="7" t="n"/>
       <c r="K4" s="7" t="n"/>
@@ -1178,7 +1188,8 @@
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>⚠ แถบแดง "ขนาดแผ่นจริงต่างจากที่เสนอลูกค้า" ขึ้นได้ปกติ เพราะใบเสนอราคาใช้ขนาด Slab มาตรฐานของวัสดุ (3.00 × 1.60 = 4.80 ตร.ม.) แต่แผ่นจริงที่เลือกคือ 2.25 ตร.ม. ระบบล็อกยอดไว้ที่ 90,000 ตามที่เสนอและเตือนเซลล์ให้แจ้งลูกค้า เป็นพฤติกรรมตามออกแบบ (ADR-079/085) ไม่ใช่ข้อผิดพลาดและไม่ห้ามการ Confirm</t>
+          <t>[แก้/เพิ่ม] รอบ 14 ต.ค. 2569 (v109.24) — แถบแดง "ขนาดแผ่นจริงต่างจากที่เสนอลูกค้า" ยังเป็นพฤติกรรมเดิม
+⚠ แถบแดง "ขนาดแผ่นจริงต่างจากที่เสนอลูกค้า" ขึ้นได้ปกติ เพราะใบเสนอราคาใช้ขนาด Slab มาตรฐานของวัสดุ (3.00 × 1.60 = 4.80 ตร.ม.) แต่แผ่นจริงที่เลือกคือ 2.25 ตร.ม. ระบบล็อกยอดไว้ที่ 90,000 ตามที่เสนอและเตือนเซลล์ให้แจ้งลูกค้า เป็นพฤติกรรมตามออกแบบ (ADR-079/085) ไม่ใช่ข้อผิดพลาดและไม่ห้ามการ Confirm</t>
         </is>
       </c>
       <c r="I5" s="7" t="n"/>
@@ -1212,12 +1223,12 @@
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>Serial = BLK-26-0037-1 ถึง BLK-26-0037-10</t>
+          <t>Serial = BLK-26-0431-1 ถึง BLK-26-0431-10</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>ใบส่งของเป็น Done จาก Stone Inventory/Stone Available Demand 10.00 Quantity 10.00 Units · ใบสั่งขาย Delivered = 10 · Slab ทั้ง 10 แผ่นเปลี่ยนสถานะเป็น Sold (ตัวอย่างจริง EG01/OUT/00107)</t>
+          <t>ใบส่งของเป็น Done จาก Stone Inventory/Stone Available Demand 10.00 Quantity 10.00 Units · ใบสั่งขาย Delivered = 10 · Slab ทั้ง 10 แผ่นเปลี่ยนสถานะเป็น Sold (ตัวอย่างจริง EG01/OUT/00332)</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
@@ -1261,7 +1272,7 @@
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>ใบแจ้งหนี้สถานะ Posted · บรรทัดสินค้า 10.00 Units ราคา 9,000.00 รวม 90,000.00 บาท · ยอดก่อน VAT 90,000.00, VAT 7% 6,300.00, รวม 96,300.00 และ Amount Due 96,300.00 · แท็ก Analytic เป็น Sale / Granite / วัสดุ / BLK-26-0037 (ตัวอย่างจริง INV/2026/00022) · ช่อง Qty (Ton) ว่างเป็นปกติสำหรับ Slab</t>
+          <t>ใบแจ้งหนี้สถานะ Posted · บรรทัดสินค้า 10.000 Units ราคา 9,000.00 รวม 90,000.00 บาท · ยอดก่อน VAT 90,000.00, VAT 7% 6,300.00, รวม 96,300.00 และ Amount Due 96,300.00 · แท็ก Analytic เป็น Sale / Granite / วัสดุ / BLK-26-0431 (ตัวอย่างจริง INV/2026/00031) · ช่อง Qty (Ton) ว่างเป็นปกติสำหรับ Slab</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
@@ -1269,7 +1280,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H7" s="7" t="n"/>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[แก้/เพิ่ม] รอบ 14 ต.ค. 2569 (v109.24) — จำนวนในใบแจ้งหนี้แสดง 3 ตำแหน่ง (10.000 Units) เพราะรอบ Block ตั้งทศนิยมจำนวนบรรทัดบิลเป็น 3 ตำแหน่งทั้งระบบ ยอดเงินไม่เปลี่ยน
+</t>
+        </is>
+      </c>
       <c r="I7" s="7" t="n"/>
       <c r="J7" s="7" t="n"/>
       <c r="K7" s="7" t="n"/>
@@ -1299,12 +1315,12 @@
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>ต้นทุน = 22.50 ตร.ม. × 540 = 12,150 (แผ่นละ 1,215)</t>
+          <t>ต้นทุน = 10 แผ่น × 1,431.375 = 14,313.73</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>เดบิต 112100 ลูกหนี้การค้า 96,300.00 · เครดิต 411100 รายได้จากการขาย 90,000.00 · เครดิต 213200 ภาษีขาย 6,300.00 · เดบิต 511110 ต้นทุนขาย (COGS) 12,150.00 · เครดิต 113120 สินค้าคงเหลือ Slab (Ready-Made) 12,150.00 · ยอดรวมสองฝั่งเท่ากัน 108,450.00</t>
+          <t>เดบิต 112100 ลูกหนี้การค้า 96,300.00 · เครดิต 411100 รายได้จากการขาย 90,000.00 · เครดิต 213200 ภาษีขาย 6,300.00 · เดบิต 511110 ต้นทุนขาย (COGS) 14,313.73 · เครดิต 113120 สินค้าคงเหลือ Slab (Ready-Made) 14,313.73 · ยอดรวมสองฝั่งเท่ากัน 110,613.73</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
@@ -1312,7 +1328,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H8" s="7" t="n"/>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[แก้/เพิ่ม] รอบ 14 ต.ค. 2569 (v109.24) — ต้นทุนขายคือต้นทุนจริงของแผ่นที่ขาย (แผ่นละ 1,431.37 จากต้นทุน Block ก้อนนั้น) ไม่ใช่ 1,215 ของรอบ 11 ต.ค.
+</t>
+        </is>
+      </c>
       <c r="I8" s="7" t="n"/>
       <c r="J8" s="7" t="n"/>
       <c r="K8" s="7" t="n"/>
@@ -1439,17 +1460,17 @@
           <t>1. เปิดใบส่งของที่ Done กดปุ่ม Return แล้วกด Return All
 2. ในใบรับคืนที่ได้ ที่แถวสินค้ากด Details
 3. กด Add a line พิมพ์ชื่อ Slab ที่คืน ใส่จำนวน 1 ทำซ้ำทีละแผ่น
-4. กด Save แล้วกด Validate</t>
+4. กด Save แล้วกด Validate เมื่อถาม Backorder เลือก No Backorder</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>แผ่นที่คืน = BLK-26-0037-9 และ BLK-26-0037-10</t>
+          <t>แผ่นที่คืน = BLK-26-0431-9 และ BLK-26-0431-10</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>ใบรับคืนเป็น Done รับจาก Demo Hotel Customer ปลายทาง Stone Inventory/Returned - Inspect เอกสารต้นทาง "Return of EG01/OUT/00107" · Demand 10.00 แต่ Quantity 2.00 และ ไม่มี Backorder เกิดขึ้น · ข้อความมุมจอ "รับเข้าสำเร็จ / Received ... (Validated successfully)" (ตัวอย่างจริง EG01/IN/00097)</t>
+          <t>ใบรับคืนเป็น Done รับจาก Demo Hotel Customer ปลายทาง Stone Inventory/Returned - Inspect เอกสารต้นทาง "Return of EG01/OUT/00332" · Demand 10.00 แต่ Quantity 2.00 และไม่มี Backorder เกิดขึ้น (ตัวอย่างจริง EG01/IN/00377)</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -1459,7 +1480,8 @@
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>ใบรับคืนไม่เลือกแผ่นไว้ให้ ผู้รับของต้องระบุเองว่าแผ่นไหนถูกคืน เพราะลูกค้าอาจคืนไม่ครบ ตัวเลือกมีเฉพาะแผ่นที่อยู่ที่ลูกค้า · ช่อง Return ตอนเปิดครั้งแรกแสดง 0.00 เป็นปกติของ Odoo ให้กด Return All</t>
+          <t>[แก้/เพิ่ม] รอบ 14 ต.ค. 2569 (v109.24) — Validate ใบรับคืนที่รับน้อยกว่า Demand ระบบถาม Backorder ให้เลือก No Backorder (รอบนี้ยืนยันว่าไม่มี error และไม่เกิด Backorder)
+ใบรับคืนไม่เลือกแผ่นไว้ให้ ผู้รับของต้องระบุเองว่าแผ่นไหนถูกคืน เพราะลูกค้าอาจคืนไม่ครบ ตัวเลือกมีเฉพาะแผ่นที่อยู่ที่ลูกค้า · ช่อง Return ตอนเปิดครั้งแรกแสดง 0.00 เป็นปกติของ Odoo ให้กด Return All · ปุ่ม Return ที่ถูกต้องคือปุ่มบนแถบสถานะ (ไม่ใช่สมาร์ทปุ่ม Returns ที่ขึ้นหลังมีใบคืนแล้ว)</t>
         </is>
       </c>
       <c r="I4" s="7" t="n"/>
@@ -1486,7 +1508,7 @@
       <c r="D5" s="7" t="inlineStr">
         <is>
           <t>1. เปิดแอป Stone Slab &gt; Slabs
-2. ใช้ตัวกรอง Pending Inspection (หรือเอาตัวกรอง Available ออกแล้วค้นหา BLK-26-0037)</t>
+2. ใช้ตัวกรอง Pending Inspection (หรือเอาตัวกรอง Available ออกแล้วค้นหา BLK-26-0431)</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
@@ -1496,7 +1518,7 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>เห็น BLK-26-0037-9 และ BLK-26-0037-10 สถานะ "Returned - Pending Inspection" (สีส้ม) ขนาด 2.50 × 0.90 × 0.020 ม. = 2.25 ตร.ม. On Hand 1.00 · ยังไม่นับเป็นของพร้อมขาย และไม่โผล่ในตัวกรอง Available</t>
+          <t>เห็นแผ่นที่คืนสถานะ "Returned - Pending Inspection" (สีส้ม) ขนาด 2.50 × 0.90 × 0.020 ม. = 2.25 ตร.ม. On Hand 1.00 (ตามเส้นทางหลัก คือ BLK-26-0431-9 และ -10 · ในภาพคือ -7 และ -8 จากใบรับคืนใบที่สอง) · ยังไม่นับเป็นของพร้อมขาย และไม่โผล่ในตัวกรอง Available</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -1506,7 +1528,7 @@
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>หน้ารายการ Slab เปิดมาพร้อมตัวกรอง Available ซึ่งซ่อนแผ่นที่รอตรวจไว้ ให้เอาตัวกรองออกหรือใช้ตัวกรอง Pending Inspection · รายการจะมีแผ่นรอตรวจของงานอื่นบนระบบทดสอบปนอยู่ด้วย ให้ดูเฉพาะแผ่นของเรา</t>
+          <t>หน้ารายการ Slab เปิดมาพร้อมตัวกรอง Available ซึ่งซ่อนแผ่นที่รอตรวจไว้ ให้เอาตัวกรองออกหรือใช้ตัวกรอง Pending Inspection · รายการจะมีแผ่นรอตรวจของงานอื่นบนระบบทดสอบปนอยู่ด้วย ให้ดูเฉพาะแผ่นของเรา · ภาพนี้ถ่ายจากใบรับคืนใบที่สอง (EG01/IN/00378: BLK-26-0431-7 และ -8) เพราะ -9 และ -10 ถูกตรวจ/ตัดทิ้งไปแล้วตอนถ่ายภาพ TC-GP-SCS-13 ถึง 14</t>
         </is>
       </c>
       <c r="I5" s="7" t="n"/>
@@ -1538,12 +1560,12 @@
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>แผ่น = BLK-26-0037-9</t>
+          <t>แผ่น = BLK-26-0431-9</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>สถานะกลับเป็น Available ที่เก็บ Stone Inventory/Stone Available · ขนาด 2.500 × 0.900 × 0.020 = 2.2500 ตร.ม. · ต้นทุน 1,215.00 บาท เท่าเดิม ราคาขาย 4,000.00 บาท/ตร.ม. (≈ 9,000 บาท/แผ่น) · ปุ่มตรวจและปุ่มตัดทิ้งหายไป และเลือกขายได้ใหม่</t>
+          <t>สถานะกลับเป็น Available ที่เก็บ Stone Inventory/Stone Available · ขนาด 2.500 × 0.900 × 0.020 = 2.2500 ตร.ม. · ต้นทุน 1,431.375 บาท เท่าเดิม ราคาขาย 4,000.00 บาท/ตร.ม. (≈ 9,000 บาท/แผ่น) · ปุ่มตรวจและปุ่มตัดทิ้งหายไป และเลือกขายได้ใหม่</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
@@ -1553,7 +1575,7 @@
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>การ์ดอาจยังเขียน "ถูกเลือกในใบขาย: S00213" หลังตรวจแล้ว เป็นแค่ประวัติของใบขายเดิม ไม่ได้กันไม่ให้ขายซ้ำ (ระบบกันเฉพาะแผ่นที่ถูกเลือกในใบเสนอราคาที่ยังเป็นร่างหรือส่งแล้ว) · การ์ดแสดง "แรงตัด 1,000 บาท" แยกจากต้นทุน 1,215 เป็นข้อมูลแสดง ไม่ได้รวมในต้นทุนขายของใบแจ้งหนี้</t>
+          <t>การ์ดอาจยังเขียน "ถูกเลือกในใบขาย: S00625" หลังตรวจแล้ว เป็นแค่ประวัติของใบขายเดิม ไม่ได้กันไม่ให้ขายซ้ำ (ระบบกันเฉพาะแผ่นที่ถูกเลือกในใบเสนอราคาที่ยังเป็นร่างหรือส่งแล้ว) · การ์ดแสดง "แรงตัด 1,000 บาท" แยกจากต้นทุน เป็นข้อมูลแสดง ไม่ได้รวมในต้นทุนขายของใบแจ้งหนี้</t>
         </is>
       </c>
       <c r="I6" s="7" t="n"/>
@@ -1586,12 +1608,12 @@
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>แผ่น = BLK-26-0037-10</t>
+          <t>แผ่น = BLK-26-0431-10</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>สถานะแผ่นเป็น Elsewhere ที่เก็บ Inventory adjustment · ระบบสร้างเอกสาร Scrap ของ Odoo สถานะ Done จำนวน 1 ย้ายจาก Returned - Inspect ไป Inventory adjustment (ตัวอย่างจริง SP/00008) · แผ่นไม่อยู่ในสต็อกขายอีก</t>
+          <t>สถานะแผ่นเป็น Elsewhere ที่เก็บ Inventory adjustment · ระบบสร้างเอกสาร Scrap ของ Odoo สถานะ Done จำนวน 1 ย้ายจาก Returned - Inspect ไป Inventory adjustment (ตัวอย่างจริง SP/00018) · แผ่นไม่อยู่ในสต็อกขายอีก</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
@@ -1601,7 +1623,7 @@
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>ทดสอบการย้ายสต็อกแล้ว (SP/00008 Done) แต่ยังไม่ได้ตรวจรายการบัญชีของการตัดทิ้ง จึงยังไม่ระบุผลบัญชีใน test case นี้</t>
+          <t>ย้ายสต็อกแล้วตัดทิ้ง (SP/00018 Done) มูลค่าสต็อกที่ตัดออก 1,431.38 บาท (ต้นทุนแผ่น) · ยังไม่ได้ตรวจรายการบัญชีของการตัดทิ้ง จึงยังไม่ระบุผลบัญชีใน test case นี้</t>
         </is>
       </c>
       <c r="I7" s="7" t="n"/>
@@ -1627,8 +1649,8 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>1. เปิดแอป Stone Slab &gt; Blocks เปิด Block ที่ใช้ตัด
-2. ดูแท็บ Slabs หรือสมาร์ทปุ่มนับจำนวนตามสถานะ</t>
+          <t>1. เปิดแอป Stone Slab &gt; Blocks เปิด Block ที่ใช้ตัด (BLK-26-0431)
+2. ดูสมาร์ทปุ่มนับจำนวนตามสถานะและการ์ดสรุป</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
@@ -1638,7 +1660,7 @@
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>Slab ทั้งหมด 60 แผ่น = Available 51 แผ่น (114.75 ตร.ม.) + Sold 8 แผ่น (18.00 ตร.ม.) + ตัดทิ้ง 1 แผ่น (2.25 ตร.ม.) · รวม 135.00 ตร.ม. ตรงกับที่ตัดได้ในใบสั่งตัด</t>
+          <t>Slab ทั้งหมด 51 แผ่น = Available 42 แผ่น (94.50 ตร.ม.) + Sold 6 แผ่น (13.50 ตร.ม.) + Returned รอตรวจ 2 แผ่น (4.50 ตร.ม. คือ -7 และ -8 จากใบรับคืนใบที่สอง) + ตัดทิ้ง 1 แผ่น (2.25 ตร.ม.) · รวม 114.75 ตร.ม. ตรงกับที่ตัดได้ในใบสั่งตัด · การ์ด Block: 42 แผ่นพร้อมขาย ขายแล้ว 6Sold 8 − ... ให้ใช้ตัวเลขตามที่ทำจริง)</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
@@ -1646,7 +1668,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H8" s="7" t="n"/>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[แก้/เพิ่ม] รอบ 14 ต.ค. 2569 (v109.24) — จำนวนแผ่นรวมเป็น 51 (ไม่ใช่ 60) เพราะหักสูญเสียเลื่อย
+</t>
+        </is>
+      </c>
       <c r="I8" s="7" t="n"/>
       <c r="J8" s="7" t="n"/>
       <c r="K8" s="7" t="n"/>

</xml_diff>